<commit_message>
Deployed 3e3cd85 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/sample-output/CDE-2018-0117_application.xlsx
+++ b/sample-output/CDE-2018-0117_application.xlsx
@@ -895,7 +895,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Application round not specified  |  Prepared: August 23, 2026  |  Readiness Grade: A (86.6/100) — this tool's own unsourced house heuristic, not a CDFI Fund evaluation</t>
+          <t>Application round not specified  |  Prepared: September 16, 2026  |  Readiness Grade: A (86.6/100) — this tool's own unsourced house heuristic, not a CDFI Fund evaluation</t>
         </is>
       </c>
     </row>
@@ -1121,15 +1121,22 @@
         </is>
       </c>
     </row>
+    <row r="26" ht="60" customHeight="1">
+      <c r="A26" s="24" t="inlineStr">
+        <is>
+          <t>READINESS NARRATIVE WITHDRAWN. This tool emits no strengths, weaknesses or recommendations from the readiness composite, and none appear in this document. It nevertheless deducted points from the grade above, and it does not deduct silently: the full component-by-component deduction table, with the reason each row is or is not a quantity the CDFI Fund also scores, is printed by the Pipeline Analyzer page of the app and by `nmtcapp analyze`. It is not repeated here, because it is an account of what this tool did to its own number rather than a finding about this application.</t>
+        </is>
+      </c>
+    </row>
     <row r="27">
       <c r="A27" s="25" t="inlineStr">
         <is>
-          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC — Generated 2026-08-23</t>
+          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC — Generated 2026-09-16</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="33">
+  <mergeCells count="34">
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="C6:D6"/>
@@ -1137,6 +1144,7 @@
     <mergeCell ref="A27:F27"/>
     <mergeCell ref="C14:D14"/>
     <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A26:F26"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="C10:D10"/>
@@ -1235,10 +1243,10 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="70" customHeight="1">
+    <row r="9" ht="84" customHeight="1">
       <c r="A9" s="28" t="inlineStr">
         <is>
-          <t>Holding those fields is not a partial answer to Question 25 and must not be read as one: the commitment is a share of QLICI DOLLARS, this package weights nothing by QLICI dollars, and a flag that enters no denominator contributes nothing to a share. Deep Distress is a strict subset of severe distress, so the severe-distress share already includes the deep-distress share. The CDE must compute both QLICI-denominated shares from its own QLICI amounts, against the Application's own area lists, before stating either commitment. (The CY 2026 NOAA is not yet published.)</t>
+          <t>Holding those fields is not a partial answer to Question 25 and must not be read as one: the commitment is a share of QLICI DOLLARS, this package weights nothing by QLICI dollars, and a flag that enters no denominator contributes nothing to a share. Deep Distress is a strict subset of severe distress, so the severe-distress share already includes the deep-distress share. The CDE must compute both QLICI-denominated shares from its own QLICI amounts, against the Application's own area lists, before stating either commitment. (Those area lists are the CY 2024-2025 Application's; the CY 2026 Allocation Application is not yet published.)</t>
         </is>
       </c>
     </row>
@@ -1263,7 +1271,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1288,39 +1296,47 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="70" customHeight="1">
+    <row r="4" ht="84" customHeight="1">
       <c r="A4" s="28" t="inlineStr">
         <is>
-          <t>WHICH ROUND THIS IS BASED ON. This tool encodes the CY 2024-2025 NMTC Allocation Application, which is the most recent PUBLISHED Application and is closed and awarded (it opened 19 Nov 2024, closed 29 Jan 2025, and was awarded 23 Dec 2025 with $10 billion in allocation authority). The CY 2026 Allocation Application and NOAA are NOT YET PUBLISHED: the CDFI Fund has announced that CY 2026 will make $5 billion available — half the prior round — and that it will publish the round's Application Materials when the round opens.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="84" customHeight="1">
+          <t>WHICH ROUND THIS IS BASED ON. This tool encodes the CY 2024-2025 NMTC Allocation Application, which is the most recent PUBLISHED Application and is closed and awarded (it opened 19 Nov 2024, closed 29 Jan 2025, and was awarded 23 Dec 2025 with $10 billion in allocation authority). THE CY 2026 ROUND HAS OPENED, BUT ITS APPLICATION HAS NOT: the CY 2026 NOAA IS PUBLISHED — Federal Register document 2026-18883, publication date September 15, 2026 — and it makes $5 billion available, with applications due 5:00 p.m. ET on November 10, 2026. The CY 2026 Allocation Application and its Application Materials are NOT YET PUBLISHED, so the instrument encoded here is still the CY 2024-2025 one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="98" customHeight="1">
       <c r="A5" s="28" t="inlineStr">
         <is>
-          <t>USE THIS, AND THEN RE-CHECK IT. The CY 2024-2025 Application is a real federal instrument and is the right basis to prepare against today; nothing here is unreliable. But it is a PROXY for the CY 2026 instrument, not that instrument, so every round-specific figure in this document must be re-verified against the CY 2026 materials once the Fund releases them — specifically: the allocation authority and the number of awards available; the CDE certification deadline for eligibility; Question 25's QLICI-denominated commitment levels, its area-type lists and its ladder; Question 22's QLICI-denominated Non-Metropolitan minimum and maximum; Question 15's product-flexibility ladder; the scoring thresholds in the Review Process.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="42" customHeight="1">
+          <t>USE THIS, AND THEN RE-CHECK IT. The CY 2024-2025 Application is a real federal instrument and is the right basis to prepare against today; nothing here is unreliable. But it is a PROXY for the CY 2026 instrument, not that instrument, so every round-specific figure in this document must be re-verified against the CY 2026 Application Materials on the day the Fund releases them — specifically: the allocation authority and the number of awards available; the CDE certification deadline for eligibility; Question 25's QLICI-denominated commitment levels, its area-type lists and its ladder; Question 22's QLICI-denominated Non-Metropolitan minimum and maximum; Question 15's product-flexibility ladder; the scoring thresholds in the Review Process.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="70" customHeight="1">
       <c r="A6" s="28" t="inlineStr">
         <is>
-          <t>SEPARATELY, AND SOONER: to be eligible to apply in CY 2026, an organization must either already be a certified CDE as of the NOAA's Federal Register publication date, or have submitted its CDE Certification Application through AMIS by 11:59 p.m. ET on August 31, 2026. That deadline is not a figure this tool computes and it does not move with anything in this document.</t>
+          <t>THE CY 2026 CDE CERTIFICATION CUTOFFS ARE SETTLED AND ONE OF THEM HAS ALREADY CLOSED. To be eligible to apply in CY 2026 an organization had EITHER to already be a certified CDE as of the NOAA's Federal Register publication date, September 15, 2026, OR to have submitted its CDE Certification Application through AMIS by 11:59 p.m. ET on August 31, 2026. Neither route is still open: the AMIS window closed on August 31, 2026, and the as-of date the NOAA sets, September 15, 2026, has arrived. An organization that did neither CANNOT APPLY IN CY 2026. There is no late filing; its next opportunity is a future round.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="84" customHeight="1">
       <c r="A7" s="28" t="inlineStr">
         <is>
-          <t>AND IF YOU ARE A PRIOR ALLOCATEE, A THIRD OBLIGATION FALLS ON THE SAME DATE: any prior Allocatee that requires action by the CDFI Fund — certifying a Subsidiary entity as a CDE, or adding a Subsidiary CDE to an Allocation Agreement — in order to meet the Qualified Equity Investment (QEI) issuance thresholds published in the CY 2026 NOAA must submit a CDE Certification Application for its Subsidiary CDE(s) through AMIS by 11:59 p.m. ET on August 31, 2026. Full eligibility information, including the QEI issuance thresholds themselves, comes with the NOAA when it publishes. Verified against cdfifund.gov on 2026-08-20.</t>
+          <t>AND IF YOU ARE A PRIOR ALLOCATEE, A THIRD OBLIGATION FELL ON THE SAME CLOSED DATE: any prior Allocatee that required action by the CDFI Fund — certifying a Subsidiary entity as a CDE, or adding a Subsidiary CDE to an Allocation Agreement — in order to meet the Qualified Equity Investment (QEI) issuance thresholds published in the CY 2026 NOAA had to submit a CDE Certification Application for its Subsidiary CDE(s) through AMIS by 11:59 p.m. ET on August 31, 2026. That date has passed. The QEI issuance thresholds themselves are in the NOAA, Federal Register document 2026-18883; this tool neither computes them nor reproduces them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="56" customHeight="1">
+      <c r="A8" s="28" t="inlineStr">
+        <is>
+          <t>THE ONLY CY 2026 DEADLINE YOU CAN STILL MISS IS THE APPLICATION DEADLINE: 5:00 p.m. ET on November 10, 2026. Every other CY 2026 date named above is already determined. It is set by the NOAA, it is not a figure this tool computes, and nothing in this document moves it. Provenance: the CY 2026 NOAA is Federal Register document 2026-18883, filed September 14, 2026 and published September 15, 2026; the absence of CY 2026 Application Materials was confirmed on September 14, 2026.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A8:F8"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A7:F7"/>
@@ -1379,7 +1395,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-08-23</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-16</t>
         </is>
       </c>
     </row>
@@ -3908,7 +3924,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-08-23</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-16</t>
         </is>
       </c>
     </row>
@@ -5605,7 +5621,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-08-23</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-16</t>
         </is>
       </c>
     </row>
@@ -6272,7 +6288,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-08-23</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-16</t>
         </is>
       </c>
     </row>
@@ -7933,7 +7949,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-08-23</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-16</t>
         </is>
       </c>
     </row>
@@ -8126,7 +8142,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-08-23</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed d1d5eba with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/sample-output/CDE-2018-0117_application.xlsx
+++ b/sample-output/CDE-2018-0117_application.xlsx
@@ -895,7 +895,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Application round not specified  |  Prepared: September 16, 2026  |  Readiness Grade: A (86.6/100) — this tool's own unsourced house heuristic, not a CDFI Fund evaluation</t>
+          <t>Application round not specified  |  Prepared: September 18, 2026  |  Readiness Grade: A (86.6/100) — this tool's own unsourced house heuristic, not a CDFI Fund evaluation</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1131,7 @@
     <row r="27">
       <c r="A27" s="25" t="inlineStr">
         <is>
-          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC — Generated 2026-09-16</t>
+          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC — Generated 2026-09-18</t>
         </is>
       </c>
     </row>
@@ -1246,7 +1246,7 @@
     <row r="9" ht="84" customHeight="1">
       <c r="A9" s="28" t="inlineStr">
         <is>
-          <t>Holding those fields is not a partial answer to Question 25 and must not be read as one: the commitment is a share of QLICI DOLLARS, this package weights nothing by QLICI dollars, and a flag that enters no denominator contributes nothing to a share. Deep Distress is a strict subset of severe distress, so the severe-distress share already includes the deep-distress share. The CDE must compute both QLICI-denominated shares from its own QLICI amounts, against the Application's own area lists, before stating either commitment. (Those area lists are the CY 2024-2025 Application's; the CY 2026 Allocation Application is not yet published.)</t>
+          <t>Holding those fields is not a partial answer to Question 25 and must not be read as one: the commitment is a share of QLICI DOLLARS, this package weights nothing by QLICI dollars, and a flag that enters no denominator contributes nothing to a share. Deep Distress is a strict subset of severe distress, so the severe-distress share already includes the deep-distress share. The CDE must compute both QLICI-denominated shares from its own QLICI amounts, against the Application's own area lists, before stating either commitment. (Those area lists are the CY 2024-2025 Application's; the CY 2026 Allocation Application's own lists must be read from that document — see the round-provenance note for where it is.)</t>
         </is>
       </c>
     </row>
@@ -1296,38 +1296,38 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="84" customHeight="1">
+    <row r="4" ht="98" customHeight="1">
       <c r="A4" s="28" t="inlineStr">
         <is>
-          <t>WHICH ROUND THIS IS BASED ON. This tool encodes the CY 2024-2025 NMTC Allocation Application, which is the most recent PUBLISHED Application and is closed and awarded (it opened 19 Nov 2024, closed 29 Jan 2025, and was awarded 23 Dec 2025 with $10 billion in allocation authority). THE CY 2026 ROUND HAS OPENED, BUT ITS APPLICATION HAS NOT: the CY 2026 NOAA IS PUBLISHED — Federal Register document 2026-18883, publication date September 15, 2026 — and it makes $5 billion available, with applications due 5:00 p.m. ET on November 10, 2026. The CY 2026 Allocation Application and its Application Materials are NOT YET PUBLISHED, so the instrument encoded here is still the CY 2024-2025 one.</t>
+          <t>WHICH ROUND THIS IS BASED ON. This tool encodes the CY 2024-2025 NMTC Allocation Application, which is closed and awarded (it opened 19 Nov 2024, closed 29 Jan 2025, and was awarded 23 Dec 2025 with $10 billion in allocation authority). THE CY 2026 ROUND HAS OPENED: the CY 2026 NOAA IS PUBLISHED — Federal Register document 2026-18883, publication date September 15, 2026 — and it makes $5 billion available, with applications due 5:00 p.m. ET on November 10, 2026. THE CY 2026 ALLOCATION APPLICATION AND ITS APPLICATION MATERIALS ARE PUBLISHED: the CDFI Fund released them on September 17, 2026 (https://www.cdfifund.gov/news/741), and this tool confirmed the Application itself on September 17, 2026. THIS TOOL STILL ENCODES THE CY 2024-2025 INSTRUMENT, which is now a proxy for a document that exists and can be read.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="98" customHeight="1">
       <c r="A5" s="28" t="inlineStr">
         <is>
-          <t>USE THIS, AND THEN RE-CHECK IT. The CY 2024-2025 Application is a real federal instrument and is the right basis to prepare against today; nothing here is unreliable. But it is a PROXY for the CY 2026 instrument, not that instrument, so every round-specific figure in this document must be re-verified against the CY 2026 Application Materials on the day the Fund releases them — specifically: the allocation authority and the number of awards available; the CDE certification deadline for eligibility; Question 25's QLICI-denominated commitment levels, its area-type lists and its ladder; Question 22's QLICI-denominated Non-Metropolitan minimum and maximum; Question 15's product-flexibility ladder; the scoring thresholds in the Review Process.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="70" customHeight="1">
+          <t>USE THIS, AND THEN RE-CHECK IT. The CY 2024-2025 Application is a real federal instrument and nothing here is unreliable. But it is a PROXY for the CY 2026 instrument, not that instrument, and that instrument is AVAILABLE NOW: every round-specific figure in this document must be re-verified against the CY 2026 Application Materials, which the CDFI Fund publishes at https://www.cdfifund.gov/programs-training/programs/new-markets-tax-credit/apply-step — specifically: the allocation authority and the number of awards available; the CDE certification deadline for eligibility; Question 25's QLICI-denominated commitment levels, its area-type lists and its ladder; Question 22's QLICI-denominated Non-Metropolitan minimum and maximum; Question 15's product-flexibility ladder; the scoring thresholds in the Review Process.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="98" customHeight="1">
       <c r="A6" s="28" t="inlineStr">
         <is>
-          <t>THE CY 2026 CDE CERTIFICATION CUTOFFS ARE SETTLED AND ONE OF THEM HAS ALREADY CLOSED. To be eligible to apply in CY 2026 an organization had EITHER to already be a certified CDE as of the NOAA's Federal Register publication date, September 15, 2026, OR to have submitted its CDE Certification Application through AMIS by 11:59 p.m. ET on August 31, 2026. Neither route is still open: the AMIS window closed on August 31, 2026, and the as-of date the NOAA sets, September 15, 2026, has arrived. An organization that did neither CANNOT APPLY IN CY 2026. There is no late filing; its next opportunity is a future round.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="84" customHeight="1">
+          <t>THE CY 2026 CDE CERTIFICATION RULE HAS TWO ROUTES, AND THE SECOND HAS A DATE IN TABLE 1 OF THE NOAA. To be eligible to apply in CY 2026 an organization must EITHER already be a certified CDE as of the NOAA's Federal Register publication date, September 15, 2026, OR submit its CDE Certification Application through AMIS by 11:59 p.m. ET on September 22, 2026. As of September 18, 2026 the AMIS route is STILL AHEAD: an organization that is not yet a certified CDE can still meet the rule by submitting its CDE Certification Application through AMIS by 11:59 p.m. ET on September 22, 2026. The NOAA adds that the CDFI Fund will not provide allocation authority to an Applicant that is not certified as a CDE. An organization that does neither CANNOT APPLY IN CY 2026. There is no late filing; its next opportunity is a future round.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="126" customHeight="1">
       <c r="A7" s="28" t="inlineStr">
         <is>
-          <t>AND IF YOU ARE A PRIOR ALLOCATEE, A THIRD OBLIGATION FELL ON THE SAME CLOSED DATE: any prior Allocatee that required action by the CDFI Fund — certifying a Subsidiary entity as a CDE, or adding a Subsidiary CDE to an Allocation Agreement — in order to meet the Qualified Equity Investment (QEI) issuance thresholds published in the CY 2026 NOAA had to submit a CDE Certification Application for its Subsidiary CDE(s) through AMIS by 11:59 p.m. ET on August 31, 2026. That date has passed. The QEI issuance thresholds themselves are in the NOAA, Federal Register document 2026-18883; this tool neither computes them nor reproduces them.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="56" customHeight="1">
+          <t>AND IF YOU ARE A PRIOR ALLOCATEE, TABLE 1 BINDS YOU ON DATES OF ITS OWN: any prior Allocatee that requires action by the CDFI Fund in order to meet the Qualified Equity Investment (QEI) issuance thresholds published in the CY 2026 NOAA must submit a CDE Certification Application for its Subsidiary CDE(s) through AMIS by 11:59 p.m. ET on September 22, 2026, and any Allocation Agreement amendment request to add Subsidiary CDEs by 11:59 p.m. ET on November 3, 2026. As of September 18, 2026 both of those dates are still ahead. The thresholds are eligibility conditions with their own deadlines, both after the application deadline: the Table 2 share of prior-round QEIs must be finalized, and the required share of them used to make QLICIs, by 11:59 p.m. ET on January 7, 2027, and those QEIs reported and QLICIs certified in AMIS by 11:59 p.m. ET on January 14, 2027. The QEI issuance thresholds themselves are in Table 2 of the NOAA, Federal Register document 2026-18883; this tool neither computes them nor reproduces them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="224" customHeight="1">
       <c r="A8" s="28" t="inlineStr">
         <is>
-          <t>THE ONLY CY 2026 DEADLINE YOU CAN STILL MISS IS THE APPLICATION DEADLINE: 5:00 p.m. ET on November 10, 2026. Every other CY 2026 date named above is already determined. It is set by the NOAA, it is not a figure this tool computes, and nothing in this document moves it. Provenance: the CY 2026 NOAA is Federal Register document 2026-18883, filed September 14, 2026 and published September 15, 2026; the absence of CY 2026 Application Materials was confirmed on September 14, 2026.</t>
+          <t>THE CY 2026 DEADLINES STILL AHEAD, COMPUTED FROM TABLE 1 OF THE NOAA AGAINST THE EASTERN DATE THIS DOCUMENT WAS GENERATED, September 18, 2026: 10 of the 10 deadlines in Table 1 are still ahead — Community Development Entity (CDE) Certification Application deadline — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS); Request to modify CDE certification service area — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS); Subsidiary CDE Certification Application for meeting Qualified Equity Investment (QEI) issuance thresholds — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS) [prior Allocatees]; CY 2026 Allocation Application Registration — 5:00 p.m. ET on October 6, 2026 (Electronically via AMIS); Amendment request to add Subsidiary CDEs to Allocation Agreements for meeting QEI issuance thresholds — 11:59 p.m. ET on November 3, 2026 (Electronically via AMIS) [prior Allocatees]; Amendment request to remove a Controlling Entity from Allocation Agreement(s) — 11:59 p.m. ET on November 3, 2026 (Electronically via AMIS) [prior Allocatees]; Last day to contact CDFI Fund staff — 5:00 p.m. ET on November 6, 2026 (Electronically via AMIS); CY 2026 Allocation Application deadline (including required Attachments) — 5:00 p.m. ET on November 10, 2026 (Electronically via AMIS); QEI Issuance and Qualified Low Income Community Investments (QLICIs) requirements deadline — 11:59 p.m. ET on January 7, 2027 (Not Applicable) [prior Allocatees]; Report QEIs and certify QLICIs deadline — 11:59 p.m. ET on January 14, 2027 (Electronically via AMIS) [prior Allocatees]. Already passed: none. Every one of these dates is set by the NOAA, none is a figure this tool computes, and nothing in this document moves them. Provenance: the CY 2026 NOAA is Federal Register document 2026-18883, filed September 14, 2026 and published September 15, 2026; the CY 2026 Application Materials were confirmed published on September 17, 2026.</t>
         </is>
       </c>
     </row>
@@ -1395,7 +1395,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-16</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-18</t>
         </is>
       </c>
     </row>
@@ -3924,7 +3924,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-16</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-18</t>
         </is>
       </c>
     </row>
@@ -5621,7 +5621,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-16</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-18</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-16</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-18</t>
         </is>
       </c>
     </row>
@@ -7949,7 +7949,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-16</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-18</t>
         </is>
       </c>
     </row>
@@ -8142,7 +8142,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-16</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed a29c983 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/sample-output/CDE-2018-0117_application.xlsx
+++ b/sample-output/CDE-2018-0117_application.xlsx
@@ -895,7 +895,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Application round not specified  |  Prepared: September 18, 2026  |  Readiness Grade: A (86.6/100) — this tool's own unsourced house heuristic, not a CDFI Fund evaluation</t>
+          <t>Application round not specified  |  Prepared: September 19, 2026  |  Readiness Grade: A (86.6/100) — this tool's own unsourced house heuristic, not a CDFI Fund evaluation</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1131,7 @@
     <row r="27">
       <c r="A27" s="25" t="inlineStr">
         <is>
-          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC — Generated 2026-09-18</t>
+          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC — Generated 2026-09-19</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1211,48 +1211,64 @@
     <row r="4" ht="84" customHeight="1">
       <c r="A4" s="28" t="inlineStr">
         <is>
-          <t>Question 25 of the CY 2024-2025 NMTC Allocation Application (printed pp. 38-41) sets both commitments, and both are measured on QLICIs — specifically on QLICIs "in terms of aggregate dollar amounts", tested for each QLICI. Question 25(a) asks for at least 85% of QLICIs in areas characterized by at least ONE of items 1-5 (Severe Distress; NMTC Native Areas; U.S. Island Areas; Non-Metropolitan Counties; Targeted Populations) or by at least TWO of items 6-12 (25% poverty / 70% median family income / 1.25x unemployment; Brownfield Sites; ARC and/or DRA Areas; Colonias Areas; Federal Medically Underserved Areas; FEMA Disaster Areas; Low-Income and Low-Access to Supermarkets).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="98" customHeight="1">
+          <t>Question 25 of the CY 2026 NMTC Allocation Application (printed pp. 36-40) sets both commitments, and both are measured on QLICIs — specifically on QLICIs "in terms of aggregate dollar amounts", tested for each QLICI. Question 25(a) asks for at least 85% of QLICIs in areas characterized by at least ONE of items 1-5 (Severe Distress; NMTC Native Areas; U.S. Island Areas; Non-Metropolitan Counties; Targeted Populations) or by at least TWO of items 6-12 (25% poverty / 70% median family income / 1.25x unemployment; Brownfield Sites; ARC and/or DRA Areas; Colonias Areas; Federal Medically Underserved Areas; FEMA Disaster Areas; Low-Income and Low-Access to Supermarkets).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="56" customHeight="1">
       <c r="A5" s="28" t="inlineStr">
         <is>
-          <t>"Multiple indicia of distress" is that two-of-seven test, applied per QLICI — not a loose notion of compounded distress and not a category of its own. Question 25(b)(i) is NOT a 20% bar. It is a selectable commitment level — 0, 5, 10, 15 or 20, and selecting 20 opens a field for any figure from 20% to 100% — over FOUR qualifying area types: Deep Distress, NMTC Native Areas, High Migration Rural Counties and U.S. Island Areas. A CDE that can honestly commit 10% selects 10 and has failed nothing; a CDE whose QLICIs sit in Native Areas, High Migration Rural Counties or Island Areas must count them, and no Deep Distress figure in this document does. The Application further states that "A QLICI that meets this commitment will also automatically meet the commitment made in Question 25(a)."</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="70" customHeight="1">
+          <t>"Multiple indicia of distress" is that two-of-seven test, applied per QLICI — not a loose notion of compounded distress and not a category of its own. Question 25(b)(i) is NOT a 20% bar. It is a selectable commitment level — 0, 5, 10, 15 or 20, and selecting 20 opens a field for any figure from 20% to 100% — over FIVE qualifying area types: Deep Distress, NMTC Native Areas, High Migration Rural Counties, U.S. Island Areas and Homeownership Cost Burden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="84" customHeight="1">
       <c r="A6" s="28" t="inlineStr">
         <is>
-          <t>Every distress share in this document is a share of QEI. nmtc-application-builder computes neither QLICI-denominated figure — it reads this pipeline's QLICI amounts only to print them in Appendix A and to check that each is no larger than its QEI — so no figure in this document answers either commitment, and none may be presented to the CDFI Fund as doing so. WHICH OF THE CDE'S QUALIFYING ROUTES ARE VISIBLE HERE: this package carries a per-project field for 6 of the 14 distinct area types Question 25 lists, and they do NOT share one provenance, so each is stated with its own.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="70" customHeight="1">
+          <t>The last of these is CONDITIONAL: a Homeownership Cost Burden tract, as designated in HUD's CHAS data, qualifies only "to the extent that Applicant's projected QLICI activities will finance the development or rehabilitation of affordable homeownership units in those tracts", and this package determines neither the CHAS designation nor whether a project's activity meets that condition. A CDE that can honestly commit 10% selects 10 and has failed nothing; a CDE whose QLICIs sit in Native Areas, High Migration Rural Counties or Island Areas, or finance affordable homeownership units in Homeownership Cost Burden tracts, must count them, and no Deep Distress figure in this document does.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="84" customHeight="1">
       <c r="A7" s="28" t="inlineStr">
         <is>
+          <t>The Application further states that "A QLICI that meets this commitment will also automatically meet the commitment made in Question 25(a)." Every distress share in this document is a share of QEI. nmtc-application-builder computes neither QLICI-denominated figure — it reads this pipeline's QLICI amounts only to print them in Appendix A and to check that each is no larger than its QEI — so no figure in this document answers either commitment, and none may be presented to the CDFI Fund as doing so. WHICH OF THE CDE'S QUALIFYING ROUTES ARE VISIBLE HERE: this package carries a per-project field for 6 of the 15 distinct area types Question 25 lists, and they do NOT share one provenance, so each is stated with its own.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="70" customHeight="1">
+      <c r="A8" s="28" t="inlineStr">
+        <is>
           <t>Severe Distress and Deep Distress: TOOL-VERIFIED — the distress level is read from the CDFI Fund eligibility table for the tract this package geocoded, and a CDE's own distress column is kept separately and labelled CDE-declared wherever it is shown. High Migration Rural Counties: CDE-DECLARED AND TOOL-VERIFIED — enrichment overwrites the CDE's declaration whenever nmtc-mapper returns a determination for the tract, so the declaration stands only where the tool reached none, and where enrichment did not run at all.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="98" customHeight="1">
-      <c r="A8" s="28" t="inlineStr">
-        <is>
-          <t>NMTC Native Areas and U.S. territory: CDE-DECLARED AND TOOL-UNVERIFIED — nothing in this package checks either one, and a Native Area determination is a spatial intersection against the Fund's CIMS map rather than a tract-keyed lookup this package could perform (U.S. territory is the CDE's own word; the Application's U.S. Island Areas is a specific list of five). Non-Metropolitan Counties: TOOL-VERIFIED AND TRI-STATE — the OMB designation is read for the same geocoded tract, and a project the lookup could not resolve is recorded as undetermined rather than as metropolitan, so no project is counted in a county type it was never determined to be in. It carries NOTHING for Targeted Populations and nothing for any of items 6-12; it computes no multi-indicia measure at all.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="84" customHeight="1">
       <c r="A9" s="28" t="inlineStr">
         <is>
-          <t>Holding those fields is not a partial answer to Question 25 and must not be read as one: the commitment is a share of QLICI DOLLARS, this package weights nothing by QLICI dollars, and a flag that enters no denominator contributes nothing to a share. Deep Distress is a strict subset of severe distress, so the severe-distress share already includes the deep-distress share. The CDE must compute both QLICI-denominated shares from its own QLICI amounts, against the Application's own area lists, before stating either commitment. (Those area lists are the CY 2024-2025 Application's; the CY 2026 Allocation Application's own lists must be read from that document — see the round-provenance note for where it is.)</t>
+          <t>NMTC Native Areas and U.S. territory: CDE-DECLARED AND TOOL-UNVERIFIED — nothing in this package checks either one, and a Native Area determination is a spatial intersection against the Fund's CIMS map rather than a tract-keyed lookup this package could perform (U.S. territory is the CDE's own word; the Application's U.S. Island Areas is a specific list of five). Non-Metropolitan Counties: TOOL-VERIFIED AND TRI-STATE — the OMB designation is read for the same geocoded tract, and a project the lookup could not resolve is recorded as undetermined rather than as metropolitan, so no project is counted in a county type it was never determined to be in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="84" customHeight="1">
+      <c r="A10" s="28" t="inlineStr">
+        <is>
+          <t>It carries NOTHING for Targeted Populations, nothing for Homeownership Cost Burden and nothing for any of items 6-12; it computes no multi-indicia measure at all. Holding those fields is not a partial answer to Question 25 and must not be read as one: the commitment is a share of QLICI DOLLARS, this package weights nothing by QLICI dollars, and a flag that enters no denominator contributes nothing to a share. Deep Distress is a strict subset of severe distress, so the severe-distress share already includes the deep-distress share. The CDE must compute both QLICI-denominated shares from its own QLICI amounts, against the Application's own area lists, before stating either commitment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="28" t="inlineStr">
+        <is>
+          <t>(The area lists above are the CY 2026 Allocation Application's, read from that document; see the round-provenance note for where it is and for which figures in this document are still the CY 2024-2025 Application's.)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="10">
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A10:F10"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A5:F5"/>
     <mergeCell ref="A9:F9"/>
@@ -1303,31 +1319,31 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="98" customHeight="1">
+    <row r="5" ht="112" customHeight="1">
       <c r="A5" s="28" t="inlineStr">
         <is>
-          <t>USE THIS, AND THEN RE-CHECK IT. The CY 2024-2025 Application is a real federal instrument and nothing here is unreliable. But it is a PROXY for the CY 2026 instrument, not that instrument, and that instrument is AVAILABLE NOW: every round-specific figure in this document must be re-verified against the CY 2026 Application Materials, which the CDFI Fund publishes at https://www.cdfifund.gov/programs-training/programs/new-markets-tax-credit/apply-step — specifically: the allocation authority and the number of awards available; the CDE certification deadline for eligibility; Question 25's QLICI-denominated commitment levels, its area-type lists and its ladder; Question 22's QLICI-denominated Non-Metropolitan minimum and maximum; Question 15's product-flexibility ladder; the scoring thresholds in the Review Process.</t>
+          <t>USE THIS, AND THEN RE-CHECK IT. The CY 2024-2025 Application is a real federal instrument and nothing here is unreliable. But it is a PROXY for the CY 2026 instrument, not that instrument, and that instrument is AVAILABLE NOW: every round-specific figure in this document must be re-verified against the CY 2026 Application Materials, which the CDFI Fund publishes at https://www.cdfifund.gov/programs-training/programs/new-markets-tax-credit/apply-step — specifically: the allocation authority and the number of awards available; the CDE certification deadline for eligibility; Question 25's QLICI-denominated commitment levels, its area-type lists and its ladder; Question 22's QLICI-denominated Non-Metropolitan minimum and maximum; Question 15's product-flexibility ladder; the scoring thresholds — as of September 17, 2026 this tool had not found a published CY 2026 Review Process, and the thresholds this document applies are the CY 2024-2025 Review Process's.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="98" customHeight="1">
       <c r="A6" s="28" t="inlineStr">
         <is>
-          <t>THE CY 2026 CDE CERTIFICATION RULE HAS TWO ROUTES, AND THE SECOND HAS A DATE IN TABLE 1 OF THE NOAA. To be eligible to apply in CY 2026 an organization must EITHER already be a certified CDE as of the NOAA's Federal Register publication date, September 15, 2026, OR submit its CDE Certification Application through AMIS by 11:59 p.m. ET on September 22, 2026. As of September 18, 2026 the AMIS route is STILL AHEAD: an organization that is not yet a certified CDE can still meet the rule by submitting its CDE Certification Application through AMIS by 11:59 p.m. ET on September 22, 2026. The NOAA adds that the CDFI Fund will not provide allocation authority to an Applicant that is not certified as a CDE. An organization that does neither CANNOT APPLY IN CY 2026. There is no late filing; its next opportunity is a future round.</t>
+          <t>THE CY 2026 CDE CERTIFICATION RULE HAS TWO ROUTES, AND THE SECOND HAS A DATE IN TABLE 1 OF THE NOAA. To be eligible to apply in CY 2026 an organization must EITHER already be a certified CDE as of the NOAA's Federal Register publication date, September 15, 2026, OR submit its CDE Certification Application through AMIS by 11:59 p.m. ET on September 22, 2026. As of September 19, 2026 the AMIS route is STILL AHEAD: an organization that is not yet a certified CDE can still meet the rule by submitting its CDE Certification Application through AMIS by 11:59 p.m. ET on September 22, 2026. The NOAA adds that the CDFI Fund will not provide allocation authority to an Applicant that is not certified as a CDE. An organization that does neither CANNOT APPLY IN CY 2026. There is no late filing; its next opportunity is a future round.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="126" customHeight="1">
       <c r="A7" s="28" t="inlineStr">
         <is>
-          <t>AND IF YOU ARE A PRIOR ALLOCATEE, TABLE 1 BINDS YOU ON DATES OF ITS OWN: any prior Allocatee that requires action by the CDFI Fund in order to meet the Qualified Equity Investment (QEI) issuance thresholds published in the CY 2026 NOAA must submit a CDE Certification Application for its Subsidiary CDE(s) through AMIS by 11:59 p.m. ET on September 22, 2026, and any Allocation Agreement amendment request to add Subsidiary CDEs by 11:59 p.m. ET on November 3, 2026. As of September 18, 2026 both of those dates are still ahead. The thresholds are eligibility conditions with their own deadlines, both after the application deadline: the Table 2 share of prior-round QEIs must be finalized, and the required share of them used to make QLICIs, by 11:59 p.m. ET on January 7, 2027, and those QEIs reported and QLICIs certified in AMIS by 11:59 p.m. ET on January 14, 2027. The QEI issuance thresholds themselves are in Table 2 of the NOAA, Federal Register document 2026-18883; this tool neither computes them nor reproduces them.</t>
+          <t>AND IF YOU ARE A PRIOR ALLOCATEE, TABLE 1 BINDS YOU ON DATES OF ITS OWN: any prior Allocatee that requires action by the CDFI Fund in order to meet the Qualified Equity Investment (QEI) issuance thresholds published in the CY 2026 NOAA must submit a CDE Certification Application for its Subsidiary CDE(s) through AMIS by 11:59 p.m. ET on September 22, 2026, and any Allocation Agreement amendment request to add Subsidiary CDEs by 11:59 p.m. ET on November 3, 2026. As of September 19, 2026 both of those dates are still ahead. The thresholds are eligibility conditions with their own deadlines, both after the application deadline: the Table 2 share of prior-round QEIs must be finalized, and the required share of them used to make QLICIs, by 11:59 p.m. ET on January 7, 2027, and those QEIs reported and QLICIs certified in AMIS by 11:59 p.m. ET on January 14, 2027. The QEI issuance thresholds themselves are in Table 2 of the NOAA, Federal Register document 2026-18883; this tool neither computes them nor reproduces them.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="224" customHeight="1">
       <c r="A8" s="28" t="inlineStr">
         <is>
-          <t>THE CY 2026 DEADLINES STILL AHEAD, COMPUTED FROM TABLE 1 OF THE NOAA AGAINST THE EASTERN DATE THIS DOCUMENT WAS GENERATED, September 18, 2026: 10 of the 10 deadlines in Table 1 are still ahead — Community Development Entity (CDE) Certification Application deadline — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS); Request to modify CDE certification service area — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS); Subsidiary CDE Certification Application for meeting Qualified Equity Investment (QEI) issuance thresholds — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS) [prior Allocatees]; CY 2026 Allocation Application Registration — 5:00 p.m. ET on October 6, 2026 (Electronically via AMIS); Amendment request to add Subsidiary CDEs to Allocation Agreements for meeting QEI issuance thresholds — 11:59 p.m. ET on November 3, 2026 (Electronically via AMIS) [prior Allocatees]; Amendment request to remove a Controlling Entity from Allocation Agreement(s) — 11:59 p.m. ET on November 3, 2026 (Electronically via AMIS) [prior Allocatees]; Last day to contact CDFI Fund staff — 5:00 p.m. ET on November 6, 2026 (Electronically via AMIS); CY 2026 Allocation Application deadline (including required Attachments) — 5:00 p.m. ET on November 10, 2026 (Electronically via AMIS); QEI Issuance and Qualified Low Income Community Investments (QLICIs) requirements deadline — 11:59 p.m. ET on January 7, 2027 (Not Applicable) [prior Allocatees]; Report QEIs and certify QLICIs deadline — 11:59 p.m. ET on January 14, 2027 (Electronically via AMIS) [prior Allocatees]. Already passed: none. Every one of these dates is set by the NOAA, none is a figure this tool computes, and nothing in this document moves them. Provenance: the CY 2026 NOAA is Federal Register document 2026-18883, filed September 14, 2026 and published September 15, 2026; the CY 2026 Application Materials were confirmed published on September 17, 2026.</t>
+          <t>THE CY 2026 DEADLINES STILL AHEAD, COMPUTED FROM TABLE 1 OF THE NOAA AGAINST THE EASTERN DATE THIS DOCUMENT WAS GENERATED, September 19, 2026: 10 of the 10 deadlines in Table 1 are still ahead — Community Development Entity (CDE) Certification Application deadline — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS); Request to modify CDE certification service area — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS); Subsidiary CDE Certification Application for meeting Qualified Equity Investment (QEI) issuance thresholds — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS) [prior Allocatees]; CY 2026 Allocation Application Registration — 5:00 p.m. ET on October 6, 2026 (Electronically via AMIS); Amendment request to add Subsidiary CDEs to Allocation Agreements for meeting QEI issuance thresholds — 11:59 p.m. ET on November 3, 2026 (Electronically via AMIS) [prior Allocatees]; Amendment request to remove a Controlling Entity from Allocation Agreement(s) — 11:59 p.m. ET on November 3, 2026 (Electronically via AMIS) [prior Allocatees]; Last day to contact CDFI Fund staff — 5:00 p.m. ET on November 6, 2026 (Electronically via AMIS); CY 2026 Allocation Application deadline (including required Attachments) — 5:00 p.m. ET on November 10, 2026 (Electronically via AMIS); QEI Issuance and Qualified Low Income Community Investments (QLICIs) requirements deadline — 11:59 p.m. ET on January 7, 2027 (Not Applicable) [prior Allocatees]; Report QEIs and certify QLICIs deadline — 11:59 p.m. ET on January 14, 2027 (Electronically via AMIS) [prior Allocatees]. Already passed: none. Every one of these dates is set by the NOAA, none is a figure this tool computes, and nothing in this document moves them. Provenance: the CY 2026 NOAA is Federal Register document 2026-18883, filed September 14, 2026 and published September 15, 2026; the CY 2026 Application Materials were confirmed published on September 17, 2026.</t>
         </is>
       </c>
     </row>
@@ -1395,7 +1411,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-18</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-19</t>
         </is>
       </c>
     </row>
@@ -3924,7 +3940,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-18</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-19</t>
         </is>
       </c>
     </row>
@@ -5621,7 +5637,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-18</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-19</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6304,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-18</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-19</t>
         </is>
       </c>
     </row>
@@ -7949,7 +7965,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-18</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-19</t>
         </is>
       </c>
     </row>
@@ -8142,7 +8158,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-18</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed ced93de with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/sample-output/CDE-2018-0117_application.xlsx
+++ b/sample-output/CDE-2018-0117_application.xlsx
@@ -895,7 +895,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Application round not specified  |  Prepared: September 19, 2026  |  Readiness Grade: A (86.6/100) — this tool's own unsourced house heuristic, not a CDFI Fund evaluation</t>
+          <t>Application round not specified  |  Prepared: September 21, 2026  |  Readiness Grade: A (86.6/100) — this tool's own unsourced house heuristic, not a CDFI Fund evaluation</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1131,7 @@
     <row r="27">
       <c r="A27" s="25" t="inlineStr">
         <is>
-          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC — Generated 2026-09-19</t>
+          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC — Generated 2026-09-21 by nmtc-application-builder v1.7.1</t>
         </is>
       </c>
     </row>
@@ -1329,21 +1329,21 @@
     <row r="6" ht="98" customHeight="1">
       <c r="A6" s="28" t="inlineStr">
         <is>
-          <t>THE CY 2026 CDE CERTIFICATION RULE HAS TWO ROUTES, AND THE SECOND HAS A DATE IN TABLE 1 OF THE NOAA. To be eligible to apply in CY 2026 an organization must EITHER already be a certified CDE as of the NOAA's Federal Register publication date, September 15, 2026, OR submit its CDE Certification Application through AMIS by 11:59 p.m. ET on September 22, 2026. As of September 19, 2026 the AMIS route is STILL AHEAD: an organization that is not yet a certified CDE can still meet the rule by submitting its CDE Certification Application through AMIS by 11:59 p.m. ET on September 22, 2026. The NOAA adds that the CDFI Fund will not provide allocation authority to an Applicant that is not certified as a CDE. An organization that does neither CANNOT APPLY IN CY 2026. There is no late filing; its next opportunity is a future round.</t>
+          <t>THE CY 2026 CDE CERTIFICATION RULE HAS TWO ROUTES, AND THE SECOND HAS A DATE IN TABLE 1 OF THE NOAA. To be eligible to apply in CY 2026 an organization must EITHER already be a certified CDE as of the NOAA's Federal Register publication date, September 15, 2026, OR submit its CDE Certification Application through AMIS by 11:59 p.m. ET on September 22, 2026. As of September 20, 2026 the AMIS route is STILL AHEAD: an organization that is not yet a certified CDE can still meet the rule by submitting its CDE Certification Application through AMIS by 11:59 p.m. ET on September 22, 2026. The NOAA adds that the CDFI Fund will not provide allocation authority to an Applicant that is not certified as a CDE. An organization that does neither CANNOT APPLY IN CY 2026. There is no late filing; its next opportunity is a future round.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="126" customHeight="1">
       <c r="A7" s="28" t="inlineStr">
         <is>
-          <t>AND IF YOU ARE A PRIOR ALLOCATEE, TABLE 1 BINDS YOU ON DATES OF ITS OWN: any prior Allocatee that requires action by the CDFI Fund in order to meet the Qualified Equity Investment (QEI) issuance thresholds published in the CY 2026 NOAA must submit a CDE Certification Application for its Subsidiary CDE(s) through AMIS by 11:59 p.m. ET on September 22, 2026, and any Allocation Agreement amendment request to add Subsidiary CDEs by 11:59 p.m. ET on November 3, 2026. As of September 19, 2026 both of those dates are still ahead. The thresholds are eligibility conditions with their own deadlines, both after the application deadline: the Table 2 share of prior-round QEIs must be finalized, and the required share of them used to make QLICIs, by 11:59 p.m. ET on January 7, 2027, and those QEIs reported and QLICIs certified in AMIS by 11:59 p.m. ET on January 14, 2027. The QEI issuance thresholds themselves are in Table 2 of the NOAA, Federal Register document 2026-18883; this tool neither computes them nor reproduces them.</t>
+          <t>AND IF YOU ARE A PRIOR ALLOCATEE, TABLE 1 BINDS YOU ON DATES OF ITS OWN: any prior Allocatee that requires action by the CDFI Fund in order to meet the Qualified Equity Investment (QEI) issuance thresholds published in the CY 2026 NOAA must submit a CDE Certification Application for its Subsidiary CDE(s) through AMIS by 11:59 p.m. ET on September 22, 2026, and any Allocation Agreement amendment request to add Subsidiary CDEs by 11:59 p.m. ET on November 3, 2026. As of September 20, 2026 both of those dates are still ahead. The thresholds are eligibility conditions with their own deadlines, both after the application deadline: the Table 2 share of prior-round QEIs must be finalized, and the required share of them used to make QLICIs, by 11:59 p.m. ET on January 7, 2027, and those QEIs reported and QLICIs certified in AMIS by 11:59 p.m. ET on January 14, 2027. The QEI issuance thresholds themselves are in Table 2 of the NOAA, Federal Register document 2026-18883; this tool neither computes them nor reproduces them.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="224" customHeight="1">
       <c r="A8" s="28" t="inlineStr">
         <is>
-          <t>THE CY 2026 DEADLINES STILL AHEAD, COMPUTED FROM TABLE 1 OF THE NOAA AGAINST THE EASTERN DATE THIS DOCUMENT WAS GENERATED, September 19, 2026: 10 of the 10 deadlines in Table 1 are still ahead — Community Development Entity (CDE) Certification Application deadline — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS); Request to modify CDE certification service area — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS); Subsidiary CDE Certification Application for meeting Qualified Equity Investment (QEI) issuance thresholds — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS) [prior Allocatees]; CY 2026 Allocation Application Registration — 5:00 p.m. ET on October 6, 2026 (Electronically via AMIS); Amendment request to add Subsidiary CDEs to Allocation Agreements for meeting QEI issuance thresholds — 11:59 p.m. ET on November 3, 2026 (Electronically via AMIS) [prior Allocatees]; Amendment request to remove a Controlling Entity from Allocation Agreement(s) — 11:59 p.m. ET on November 3, 2026 (Electronically via AMIS) [prior Allocatees]; Last day to contact CDFI Fund staff — 5:00 p.m. ET on November 6, 2026 (Electronically via AMIS); CY 2026 Allocation Application deadline (including required Attachments) — 5:00 p.m. ET on November 10, 2026 (Electronically via AMIS); QEI Issuance and Qualified Low Income Community Investments (QLICIs) requirements deadline — 11:59 p.m. ET on January 7, 2027 (Not Applicable) [prior Allocatees]; Report QEIs and certify QLICIs deadline — 11:59 p.m. ET on January 14, 2027 (Electronically via AMIS) [prior Allocatees]. Already passed: none. Every one of these dates is set by the NOAA, none is a figure this tool computes, and nothing in this document moves them. Provenance: the CY 2026 NOAA is Federal Register document 2026-18883, filed September 14, 2026 and published September 15, 2026; the CY 2026 Application Materials were confirmed published on September 17, 2026.</t>
+          <t>THE CY 2026 DEADLINES STILL AHEAD, COMPUTED FROM TABLE 1 OF THE NOAA AGAINST THE EASTERN DATE THIS DOCUMENT WAS GENERATED, September 20, 2026: 10 of the 10 deadlines in Table 1 are still ahead — Community Development Entity (CDE) Certification Application deadline — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS); Request to modify CDE certification service area — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS); Subsidiary CDE Certification Application for meeting Qualified Equity Investment (QEI) issuance thresholds — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS) [prior Allocatees]; CY 2026 Allocation Application Registration — 5:00 p.m. ET on October 6, 2026 (Electronically via AMIS); Amendment request to add Subsidiary CDEs to Allocation Agreements for meeting QEI issuance thresholds — 11:59 p.m. ET on November 3, 2026 (Electronically via AMIS) [prior Allocatees]; Amendment request to remove a Controlling Entity from Allocation Agreement(s) — 11:59 p.m. ET on November 3, 2026 (Electronically via AMIS) [prior Allocatees]; Last day to contact CDFI Fund staff — 5:00 p.m. ET on November 6, 2026 (Electronically via AMIS); CY 2026 Allocation Application deadline (including required Attachments) — 5:00 p.m. ET on November 10, 2026 (Electronically via AMIS); QEI Issuance and Qualified Low Income Community Investments (QLICIs) requirements deadline — 11:59 p.m. ET on January 7, 2027 (Not Applicable) [prior Allocatees]; Report QEIs and certify QLICIs deadline — 11:59 p.m. ET on January 14, 2027 (Electronically via AMIS) [prior Allocatees]. Already passed: none. Every one of these dates is set by the NOAA, none is a figure this tool computes, and nothing in this document moves them. Provenance: the CY 2026 NOAA is Federal Register document 2026-18883, filed September 14, 2026 and published September 15, 2026; the CY 2026 Application Materials were confirmed published on September 17, 2026.</t>
         </is>
       </c>
     </row>
@@ -1411,7 +1411,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-19</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-21</t>
         </is>
       </c>
     </row>
@@ -3940,7 +3940,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-19</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-21</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-19</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-21</t>
         </is>
       </c>
     </row>
@@ -6304,7 +6304,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-19</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-21</t>
         </is>
       </c>
     </row>
@@ -7965,7 +7965,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-19</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-21</t>
         </is>
       </c>
     </row>
@@ -8158,7 +8158,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-19</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed cd61870 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/sample-output/CDE-2018-0117_application.xlsx
+++ b/sample-output/CDE-2018-0117_application.xlsx
@@ -895,7 +895,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Application round not specified  |  Prepared: September 25, 2026  |  Readiness Grade: A (86.6/100) — this tool's own unsourced house heuristic, not a CDFI Fund evaluation</t>
+          <t>Application round not specified  |  Prepared: September 29, 2026  |  Readiness Grade: A (86.6/100) — this tool's own unsourced house heuristic, not a CDFI Fund evaluation</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1131,7 @@
     <row r="27">
       <c r="A27" s="25" t="inlineStr">
         <is>
-          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC — Generated 2026-09-25 by nmtc-application-builder v1.7.1</t>
+          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC — Generated 2026-09-29 by nmtc-application-builder v1.7.2</t>
         </is>
       </c>
     </row>
@@ -1329,21 +1329,21 @@
     <row r="6" ht="98" customHeight="1">
       <c r="A6" s="28" t="inlineStr">
         <is>
-          <t>THE CY 2026 CDE CERTIFICATION RULE HAS TWO ROUTES, AND THE SECOND HAS A DATE IN TABLE 1 OF THE NOAA. To be eligible to apply in CY 2026 an organization must EITHER already be a certified CDE as of the NOAA's Federal Register publication date, September 15, 2026, OR submit its CDE Certification Application through AMIS by 11:59 p.m. ET on September 22, 2026. As of September 24, 2026 the AMIS route has CLOSED: the window shut at 11:59 p.m. ET on September 22, 2026, and the as-of date, September 15, 2026, has passed. The NOAA adds that the CDFI Fund will not provide allocation authority to an Applicant that is not certified as a CDE. An organization that did neither CANNOT APPLY IN CY 2026. There is no late filing; its next opportunity is a future round.</t>
+          <t>THE CY 2026 CDE CERTIFICATION RULE HAS TWO ROUTES, AND THE SECOND HAS A DATE IN TABLE 1 OF THE NOAA. To be eligible to apply in CY 2026 an organization must EITHER already be a certified CDE as of the NOAA's Federal Register publication date, September 15, 2026, OR submit its CDE Certification Application through AMIS by 11:59 p.m. ET on September 22, 2026. As of September 29, 2026 the AMIS route has CLOSED: the window shut at 11:59 p.m. ET on September 22, 2026, and the as-of date, September 15, 2026, has passed. The NOAA adds that the CDFI Fund will not provide allocation authority to an Applicant that is not certified as a CDE. An organization that did neither CANNOT APPLY IN CY 2026. There is no late filing; its next opportunity is a future round.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="126" customHeight="1">
       <c r="A7" s="28" t="inlineStr">
         <is>
-          <t>AND IF YOU ARE A PRIOR ALLOCATEE, TABLE 1 BINDS YOU ON DATES OF ITS OWN: any prior Allocatee that requires action by the CDFI Fund in order to meet the Qualified Equity Investment (QEI) issuance thresholds published in the CY 2026 NOAA must submit a CDE Certification Application for its Subsidiary CDE(s) through AMIS by 11:59 p.m. ET on September 22, 2026, and any Allocation Agreement amendment request to add Subsidiary CDEs by 11:59 p.m. ET on November 3, 2026. As of September 24, 2026 the Subsidiary CDE certification date has passed and the amendment date is still ahead. The thresholds are eligibility conditions with their own deadlines, both after the application deadline: the Table 2 share of prior-round QEIs must be finalized, and the required share of them used to make QLICIs, by 11:59 p.m. ET on January 7, 2027, and those QEIs reported and QLICIs certified in AMIS by 11:59 p.m. ET on January 14, 2027. The QEI issuance thresholds themselves are in Table 2 of the NOAA, Federal Register document 2026-18883; this tool neither computes them nor reproduces them.</t>
+          <t>AND IF YOU ARE A PRIOR ALLOCATEE, TABLE 1 BINDS YOU ON DATES OF ITS OWN: any prior Allocatee that requires action by the CDFI Fund in order to meet the Qualified Equity Investment (QEI) issuance thresholds published in the CY 2026 NOAA must submit a CDE Certification Application for its Subsidiary CDE(s) through AMIS by 11:59 p.m. ET on September 22, 2026, and any Allocation Agreement amendment request to add Subsidiary CDEs by 11:59 p.m. ET on November 3, 2026. As of September 29, 2026 the Subsidiary CDE certification date has passed and the amendment date is still ahead. The thresholds are eligibility conditions with their own deadlines, both after the application deadline: the Table 2 share of prior-round QEIs must be finalized, and the required share of them used to make QLICIs, by 11:59 p.m. ET on January 7, 2027, and those QEIs reported and QLICIs certified in AMIS by 11:59 p.m. ET on January 14, 2027. The QEI issuance thresholds themselves are in Table 2 of the NOAA, Federal Register document 2026-18883; this tool neither computes them nor reproduces them.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="224" customHeight="1">
       <c r="A8" s="28" t="inlineStr">
         <is>
-          <t>THE CY 2026 DEADLINES STILL AHEAD, COMPUTED FROM TABLE 1 OF THE NOAA AGAINST THE EASTERN DATE THIS DOCUMENT WAS GENERATED, September 24, 2026: 7 of the 10 deadlines in Table 1 are still ahead — CY 2026 Allocation Application Registration — 5:00 p.m. ET on October 6, 2026 (Electronically via AMIS); Amendment request to add Subsidiary CDEs to Allocation Agreements for meeting QEI issuance thresholds — 11:59 p.m. ET on November 3, 2026 (Electronically via AMIS) [prior Allocatees]; Amendment request to remove a Controlling Entity from Allocation Agreement(s) — 11:59 p.m. ET on November 3, 2026 (Electronically via AMIS) [prior Allocatees]; Last day to contact CDFI Fund staff — 5:00 p.m. ET on November 6, 2026 (Electronically via AMIS); CY 2026 Allocation Application deadline (including required Attachments) — 5:00 p.m. ET on November 10, 2026 (Electronically via AMIS); QEI Issuance and Qualified Low Income Community Investments (QLICIs) requirements deadline — 11:59 p.m. ET on January 7, 2027 (Not Applicable) [prior Allocatees]; Report QEIs and certify QLICIs deadline — 11:59 p.m. ET on January 14, 2027 (Electronically via AMIS) [prior Allocatees]. Already passed: Community Development Entity (CDE) Certification Application deadline — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS); Request to modify CDE certification service area — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS); Subsidiary CDE Certification Application for meeting Qualified Equity Investment (QEI) issuance thresholds — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS) [prior Allocatees]. Every one of these dates is set by the NOAA, none is a figure this tool computes, and nothing in this document moves them. Provenance: the CY 2026 NOAA is Federal Register document 2026-18883, filed September 14, 2026 and published September 15, 2026; the CY 2026 Application Materials were confirmed published on September 17, 2026.</t>
+          <t>THE CY 2026 DEADLINES STILL AHEAD, COMPUTED FROM TABLE 1 OF THE NOAA AGAINST THE EASTERN DATE THIS DOCUMENT WAS GENERATED, September 29, 2026: 7 of the 10 deadlines in Table 1 are still ahead — CY 2026 Allocation Application Registration — 5:00 p.m. ET on October 6, 2026 (Electronically via AMIS); Amendment request to add Subsidiary CDEs to Allocation Agreements for meeting QEI issuance thresholds — 11:59 p.m. ET on November 3, 2026 (Electronically via AMIS) [prior Allocatees]; Amendment request to remove a Controlling Entity from Allocation Agreement(s) — 11:59 p.m. ET on November 3, 2026 (Electronically via AMIS) [prior Allocatees]; Last day to contact CDFI Fund staff — 5:00 p.m. ET on November 6, 2026 (Electronically via AMIS); CY 2026 Allocation Application deadline (including required Attachments) — 5:00 p.m. ET on November 10, 2026 (Electronically via AMIS); QEI Issuance and Qualified Low Income Community Investments (QLICIs) requirements deadline — 11:59 p.m. ET on January 7, 2027 (Not Applicable) [prior Allocatees]; Report QEIs and certify QLICIs deadline — 11:59 p.m. ET on January 14, 2027 (Electronically via AMIS) [prior Allocatees]. Already passed: Community Development Entity (CDE) Certification Application deadline — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS); Request to modify CDE certification service area — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS); Subsidiary CDE Certification Application for meeting Qualified Equity Investment (QEI) issuance thresholds — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS) [prior Allocatees]. Every one of these dates is set by the NOAA, none is a figure this tool computes, and nothing in this document moves them. Provenance: the CY 2026 NOAA is Federal Register document 2026-18883, filed September 14, 2026 and published September 15, 2026; the CY 2026 Application Materials were confirmed published on September 17, 2026.</t>
         </is>
       </c>
     </row>
@@ -1411,7 +1411,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-25</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-29</t>
         </is>
       </c>
     </row>
@@ -3940,7 +3940,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-25</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-29</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-25</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-29</t>
         </is>
       </c>
     </row>
@@ -6304,7 +6304,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-25</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-29</t>
         </is>
       </c>
     </row>
@@ -7965,7 +7965,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-25</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-29</t>
         </is>
       </c>
     </row>
@@ -8158,7 +8158,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-25</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed eecf16b with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/sample-output/CDE-2018-0117_application.xlsx
+++ b/sample-output/CDE-2018-0117_application.xlsx
@@ -895,7 +895,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Application round not specified  |  Prepared: September 29, 2026  |  Readiness Grade: A (86.6/100) — this tool's own unsourced house heuristic, not a CDFI Fund evaluation</t>
+          <t>Application round not specified  |  Prepared: October 09, 2026  |  Readiness Grade: A (86.6/100) — this tool's own unsourced house heuristic, not a CDFI Fund evaluation</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1131,7 @@
     <row r="27">
       <c r="A27" s="25" t="inlineStr">
         <is>
-          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC — Generated 2026-09-29 by nmtc-application-builder v1.7.2</t>
+          <t>CONFIDENTIAL — Riverbend Community Capital CDE, LLC — NMTC — Generated 2026-10-09 by nmtc-application-builder v1.7.3</t>
         </is>
       </c>
     </row>
@@ -1322,28 +1322,28 @@
     <row r="5" ht="112" customHeight="1">
       <c r="A5" s="28" t="inlineStr">
         <is>
-          <t>USE THIS, AND THEN RE-CHECK IT. The CY 2024-2025 Application is a real federal instrument and nothing here is unreliable. But it is a PROXY for the CY 2026 instrument, not that instrument, and that instrument is AVAILABLE NOW: every round-specific figure in this document must be re-verified against the CY 2026 Application Materials, which the CDFI Fund publishes at https://www.cdfifund.gov/programs-training/programs/new-markets-tax-credit/apply-step — specifically: the allocation authority and the number of awards available; the CDE certification deadline for eligibility; Question 25's QLICI-denominated commitment levels, its area-type lists and its ladder; Question 22's QLICI-denominated Non-Metropolitan minimum and maximum; Question 15's product-flexibility ladder; the scoring thresholds — as of September 17, 2026 this tool had not found a published CY 2026 Review Process, and the thresholds this document applies are the CY 2024-2025 Review Process's.</t>
+          <t>USE THIS, AND THEN RE-CHECK IT. The CY 2024-2025 Application is a real federal instrument and nothing here is unreliable. But it is a PROXY for the CY 2026 instrument, not that instrument, and that instrument is AVAILABLE NOW: every round-specific figure in this document must be re-verified against the CY 2026 Application Materials, which the CDFI Fund publishes at https://www.cdfifund.gov/programs-training/programs/new-markets-tax-credit/apply-step — specifically: the allocation authority and the number of awards available; the CDE certification deadline for eligibility; Question 25's QLICI-denominated commitment levels, its area-type lists and its ladder; Question 22's QLICI-denominated Non-Metropolitan minimum and maximum; Question 15's product-flexibility ladder; the scoring thresholds — as of October 8, 2026 this tool had not found a published CY 2026 Review Process, and the thresholds this document applies are the CY 2024-2025 Review Process's.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="98" customHeight="1">
       <c r="A6" s="28" t="inlineStr">
         <is>
-          <t>THE CY 2026 CDE CERTIFICATION RULE HAS TWO ROUTES, AND THE SECOND HAS A DATE IN TABLE 1 OF THE NOAA. To be eligible to apply in CY 2026 an organization must EITHER already be a certified CDE as of the NOAA's Federal Register publication date, September 15, 2026, OR submit its CDE Certification Application through AMIS by 11:59 p.m. ET on September 22, 2026. As of September 29, 2026 the AMIS route has CLOSED: the window shut at 11:59 p.m. ET on September 22, 2026, and the as-of date, September 15, 2026, has passed. The NOAA adds that the CDFI Fund will not provide allocation authority to an Applicant that is not certified as a CDE. An organization that did neither CANNOT APPLY IN CY 2026. There is no late filing; its next opportunity is a future round.</t>
+          <t>THE CY 2026 CDE CERTIFICATION RULE HAS TWO ROUTES, AND THE SECOND HAS A DATE IN TABLE 1 OF THE NOAA. To be eligible to apply in CY 2026 an organization must EITHER already be a certified CDE as of the NOAA's Federal Register publication date, September 15, 2026, OR submit its CDE Certification Application through AMIS by 11:59 p.m. ET on September 22, 2026. As of October 8, 2026 the AMIS route has CLOSED: the window shut at 11:59 p.m. ET on September 22, 2026, and the as-of date, September 15, 2026, has passed. The NOAA adds that the CDFI Fund will not provide allocation authority to an Applicant that is not certified as a CDE. An organization that did neither CANNOT APPLY IN CY 2026. There is no late filing; its next opportunity is a future round.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="126" customHeight="1">
       <c r="A7" s="28" t="inlineStr">
         <is>
-          <t>AND IF YOU ARE A PRIOR ALLOCATEE, TABLE 1 BINDS YOU ON DATES OF ITS OWN: any prior Allocatee that requires action by the CDFI Fund in order to meet the Qualified Equity Investment (QEI) issuance thresholds published in the CY 2026 NOAA must submit a CDE Certification Application for its Subsidiary CDE(s) through AMIS by 11:59 p.m. ET on September 22, 2026, and any Allocation Agreement amendment request to add Subsidiary CDEs by 11:59 p.m. ET on November 3, 2026. As of September 29, 2026 the Subsidiary CDE certification date has passed and the amendment date is still ahead. The thresholds are eligibility conditions with their own deadlines, both after the application deadline: the Table 2 share of prior-round QEIs must be finalized, and the required share of them used to make QLICIs, by 11:59 p.m. ET on January 7, 2027, and those QEIs reported and QLICIs certified in AMIS by 11:59 p.m. ET on January 14, 2027. The QEI issuance thresholds themselves are in Table 2 of the NOAA, Federal Register document 2026-18883; this tool neither computes them nor reproduces them.</t>
+          <t>AND IF YOU ARE A PRIOR ALLOCATEE, TABLE 1 BINDS YOU ON DATES OF ITS OWN: any prior Allocatee that requires action by the CDFI Fund in order to meet the Qualified Equity Investment (QEI) issuance thresholds published in the CY 2026 NOAA must submit a CDE Certification Application for its Subsidiary CDE(s) through AMIS by 11:59 p.m. ET on September 22, 2026, and any Allocation Agreement amendment request to add Subsidiary CDEs by 11:59 p.m. ET on November 3, 2026. As of October 8, 2026 the Subsidiary CDE certification date has passed and the amendment date is still ahead. The thresholds are eligibility conditions with their own deadlines, both after the application deadline: the Table 2 share of prior-round QEIs must be finalized, and the required share of them used to make QLICIs, by 11:59 p.m. ET on January 7, 2027, and those QEIs reported and QLICIs certified in AMIS by 11:59 p.m. ET on January 14, 2027. The QEI issuance thresholds themselves are in Table 2 of the NOAA, Federal Register document 2026-18883; this tool neither computes them nor reproduces them.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="224" customHeight="1">
       <c r="A8" s="28" t="inlineStr">
         <is>
-          <t>THE CY 2026 DEADLINES STILL AHEAD, COMPUTED FROM TABLE 1 OF THE NOAA AGAINST THE EASTERN DATE THIS DOCUMENT WAS GENERATED, September 29, 2026: 7 of the 10 deadlines in Table 1 are still ahead — CY 2026 Allocation Application Registration — 5:00 p.m. ET on October 6, 2026 (Electronically via AMIS); Amendment request to add Subsidiary CDEs to Allocation Agreements for meeting QEI issuance thresholds — 11:59 p.m. ET on November 3, 2026 (Electronically via AMIS) [prior Allocatees]; Amendment request to remove a Controlling Entity from Allocation Agreement(s) — 11:59 p.m. ET on November 3, 2026 (Electronically via AMIS) [prior Allocatees]; Last day to contact CDFI Fund staff — 5:00 p.m. ET on November 6, 2026 (Electronically via AMIS); CY 2026 Allocation Application deadline (including required Attachments) — 5:00 p.m. ET on November 10, 2026 (Electronically via AMIS); QEI Issuance and Qualified Low Income Community Investments (QLICIs) requirements deadline — 11:59 p.m. ET on January 7, 2027 (Not Applicable) [prior Allocatees]; Report QEIs and certify QLICIs deadline — 11:59 p.m. ET on January 14, 2027 (Electronically via AMIS) [prior Allocatees]. Already passed: Community Development Entity (CDE) Certification Application deadline — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS); Request to modify CDE certification service area — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS); Subsidiary CDE Certification Application for meeting Qualified Equity Investment (QEI) issuance thresholds — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS) [prior Allocatees]. Every one of these dates is set by the NOAA, none is a figure this tool computes, and nothing in this document moves them. Provenance: the CY 2026 NOAA is Federal Register document 2026-18883, filed September 14, 2026 and published September 15, 2026; the CY 2026 Application Materials were confirmed published on September 17, 2026.</t>
+          <t>THE CY 2026 DEADLINES STILL AHEAD, COMPUTED FROM TABLE 1 OF THE NOAA AGAINST THE EASTERN DATE THIS DOCUMENT WAS GENERATED, October 8, 2026: 6 of the 10 deadlines in Table 1 are still ahead — Amendment request to add Subsidiary CDEs to Allocation Agreements for meeting QEI issuance thresholds — 11:59 p.m. ET on November 3, 2026 (Electronically via AMIS) [prior Allocatees]; Amendment request to remove a Controlling Entity from Allocation Agreement(s) — 11:59 p.m. ET on November 3, 2026 (Electronically via AMIS) [prior Allocatees]; Last day to contact CDFI Fund staff — 5:00 p.m. ET on November 6, 2026 (Electronically via AMIS); CY 2026 Allocation Application deadline (including required Attachments) — 5:00 p.m. ET on November 10, 2026 (Electronically via AMIS); QEI Issuance and Qualified Low Income Community Investments (QLICIs) requirements deadline — 11:59 p.m. ET on January 7, 2027 (Not Applicable) [prior Allocatees]; Report QEIs and certify QLICIs deadline — 11:59 p.m. ET on January 14, 2027 (Electronically via AMIS) [prior Allocatees]. Already passed: Community Development Entity (CDE) Certification Application deadline — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS); Request to modify CDE certification service area — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS); Subsidiary CDE Certification Application for meeting Qualified Equity Investment (QEI) issuance thresholds — 11:59 p.m. ET on September 22, 2026 (Electronically via AMIS) [prior Allocatees]; CY 2026 Allocation Application Registration — 5:00 p.m. ET on October 6, 2026 (Electronically via AMIS). Every one of these dates is set by the NOAA, none is a figure this tool computes, and nothing in this document moves them. Provenance: the CY 2026 NOAA is Federal Register document 2026-18883, filed September 14, 2026 and published September 15, 2026; the CY 2026 Application Materials were confirmed published on October 8, 2026.</t>
         </is>
       </c>
     </row>
@@ -1411,7 +1411,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-29</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-10-09</t>
         </is>
       </c>
     </row>
@@ -3940,7 +3940,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-29</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-10-09</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-29</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-10-09</t>
         </is>
       </c>
     </row>
@@ -6304,7 +6304,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-29</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-10-09</t>
         </is>
       </c>
     </row>
@@ -7965,7 +7965,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-29</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-10-09</t>
         </is>
       </c>
     </row>
@@ -8158,7 +8158,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-09-29</t>
+          <t>Riverbend Community Capital CDE, LLC  |  Application round not specified  |  Generated 2026-10-09</t>
         </is>
       </c>
     </row>

</xml_diff>